<commit_message>
Recruitment - search vacancy valid test related page and actions added
</commit_message>
<xml_diff>
--- a/PROJECT_OHRM/test_data/vacancy_data.xlsx
+++ b/PROJECT_OHRM/test_data/vacancy_data.xlsx
@@ -29,9 +29,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>VacancyName</t>
+  </si>
+  <si>
+    <t>Job title</t>
   </si>
   <si>
     <t>HiringManager</t>
@@ -40,7 +43,10 @@
     <t>Marketing</t>
   </si>
   <si>
-    <t>J</t>
+    <t>A</t>
+  </si>
+  <si>
+    <t>John</t>
   </si>
 </sst>
 </file>
@@ -1002,23 +1008,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="1"/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improved the locators and added the correct file path for screeenshots
</commit_message>
<xml_diff>
--- a/PROJECT_OHRM/test_data/vacancy_data.xlsx
+++ b/PROJECT_OHRM/test_data/vacancy_data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6800"/>
+    <workbookView windowWidth="19200" windowHeight="6200"/>
   </bookViews>
   <sheets>
     <sheet name="AddVacancy" sheetId="1" r:id="rId1"/>
@@ -29,21 +29,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>VacancyName</t>
-  </si>
-  <si>
-    <t>Job title</t>
   </si>
   <si>
     <t>HiringManager</t>
   </si>
   <si>
     <t>Marketing</t>
-  </si>
-  <si>
-    <t>A</t>
   </si>
   <si>
     <t>John</t>
@@ -1008,29 +1002,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="2"/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="1"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>